<commit_message>
Upload FTR Calculations 2026.xlsx via dashboard admin
</commit_message>
<xml_diff>
--- a/data/raw/FTR Calculations 2026.xlsx
+++ b/data/raw/FTR Calculations 2026.xlsx
@@ -9,7 +9,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\FTR Manufacturing- 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{440D13B2-829C-4D75-A664-FCAA283FE2EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{598F05B7-9B53-4053-8613-37E67DED7FD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="601" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21917,11 +21917,12 @@
       <sheetName val="Chart1"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
       <sheetData sheetId="6">
         <row r="172">
           <cell r="I172">
@@ -21994,13 +21995,13 @@
             <v>1</v>
           </cell>
           <cell r="E1752">
-            <v>0.44444444444444442</v>
+            <v>0.41176470588235292</v>
           </cell>
           <cell r="G1752">
-            <v>0.91304347826086951</v>
+            <v>0.93333333333333335</v>
           </cell>
           <cell r="I1752">
-            <v>0.44444444444444442</v>
+            <v>0.41176470588235292</v>
           </cell>
         </row>
       </sheetData>
@@ -22087,26 +22088,26 @@
         </row>
         <row r="505">
           <cell r="D505">
-            <v>0.8</v>
+            <v>0.83333333333333337</v>
           </cell>
           <cell r="G505">
             <v>1</v>
           </cell>
-          <cell r="I505">
-            <v>1</v>
+          <cell r="I505" t="e">
+            <v>#DIV/0!</v>
           </cell>
           <cell r="K505">
             <v>1</v>
           </cell>
           <cell r="M505">
-            <v>1</v>
+            <v>0.75</v>
           </cell>
           <cell r="P505">
-            <v>0.66666666666666663</v>
+            <v>0.5</v>
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="8"/>
+      <sheetData sheetId="8" refreshError="1"/>
       <sheetData sheetId="9">
         <row r="515">
           <cell r="D515">
@@ -22350,13 +22351,13 @@
             <v>1</v>
           </cell>
           <cell r="F631">
-            <v>0.8571428571428571</v>
+            <v>0.88888888888888884</v>
           </cell>
           <cell r="H631">
             <v>1</v>
           </cell>
           <cell r="L631">
-            <v>0.8571428571428571</v>
+            <v>0.88888888888888884</v>
           </cell>
         </row>
       </sheetData>
@@ -22519,7 +22520,7 @@
             <v>1</v>
           </cell>
           <cell r="F624">
-            <v>1</v>
+            <v>0.77777777777777779</v>
           </cell>
           <cell r="H624">
             <v>1</v>
@@ -22528,11 +22529,12 @@
             <v>1</v>
           </cell>
           <cell r="L624">
-            <v>1</v>
+            <v>0.77777777777777779</v>
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="12"/>
+      <sheetData sheetId="12" refreshError="1"/>
+      <sheetData sheetId="13" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -34382,7 +34384,7 @@
       </c>
       <c r="L2" s="51">
         <f>'[1]FTR Brewhouse'!$I$1752</f>
-        <v>0.44444444444444442</v>
+        <v>0.41176470588235292</v>
       </c>
       <c r="M2" s="51">
         <f>'[2]FTR Brewhouse'!$I$504</f>
@@ -34502,7 +34504,7 @@
       </c>
       <c r="L4" s="54">
         <f>'[1]FTR Brewhouse'!$E$1752</f>
-        <v>0.44444444444444442</v>
+        <v>0.41176470588235292</v>
       </c>
       <c r="M4" s="54">
         <f>'[2]FTR Brewhouse'!$E$504</f>
@@ -34562,7 +34564,7 @@
       </c>
       <c r="L5" s="54">
         <f>'[1]FTR Brewhouse'!$G$1752</f>
-        <v>0.91304347826086951</v>
+        <v>0.93333333333333335</v>
       </c>
       <c r="M5" s="54">
         <f>'[2]FTR Brewhouse'!$G$504</f>
@@ -34669,7 +34671,7 @@
       </c>
       <c r="L8" s="51">
         <f>'[1]FTR Fermentation'!$P$505</f>
-        <v>0.66666666666666663</v>
+        <v>0.5</v>
       </c>
       <c r="M8" s="51">
         <f>'[3]FTR Fermentation'!$P$552</f>
@@ -34729,7 +34731,7 @@
       </c>
       <c r="L9" s="54">
         <f>'[1]FTR Fermentation'!$D$505</f>
-        <v>0.8</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="M9" s="54">
         <f>'[3]FTR Fermentation'!$D$552</f>
@@ -34909,7 +34911,7 @@
       </c>
       <c r="L12" s="54">
         <f>'[1]FTR Fermentation'!$M$505</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="M12" s="54">
         <f>'[3]FTR Fermentation'!$M$552</f>
@@ -34967,9 +34969,9 @@
         <f>'[1]FTR Fermentation'!$I$457</f>
         <v>1</v>
       </c>
-      <c r="L13" s="54">
+      <c r="L13" s="54" t="e">
         <f>'[1]FTR Fermentation'!$I$505</f>
-        <v>1</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="M13" s="54">
         <f>'[3]FTR Fermentation'!$I$552</f>
@@ -35505,7 +35507,7 @@
       </c>
       <c r="L24" s="51">
         <f>'[1]FTR Packaging'!$L$631</f>
-        <v>0.8571428571428571</v>
+        <v>0.88888888888888884</v>
       </c>
       <c r="M24" s="51">
         <f>'[3]FTR Packaging'!$L$664</f>
@@ -35565,7 +35567,7 @@
       </c>
       <c r="L25" s="54">
         <f>'[1]FTR Packaging'!$F$631</f>
-        <v>0.8571428571428571</v>
+        <v>0.88888888888888884</v>
       </c>
       <c r="M25" s="54">
         <f>'[3]FTR Packaging'!$F$664</f>
@@ -35745,7 +35747,7 @@
       </c>
       <c r="L28" s="52">
         <f>'[1]FTR Packaging'!$L$631</f>
-        <v>0.8571428571428571</v>
+        <v>0.88888888888888884</v>
       </c>
       <c r="M28" s="52">
         <f>'[3]FTR Packaging'!$L$664</f>
@@ -36044,7 +36046,7 @@
       </c>
       <c r="L36" s="51">
         <f>'[1]FTR Finished Product'!$L$624</f>
-        <v>1</v>
+        <v>0.77777777777777779</v>
       </c>
       <c r="M36" s="51">
         <f>'[2]FTR Finished Product'!$L$195</f>
@@ -36164,7 +36166,7 @@
       </c>
       <c r="L38" s="57">
         <f>'[1]FTR Finished Product'!$F$624</f>
-        <v>1</v>
+        <v>0.77777777777777779</v>
       </c>
       <c r="M38" s="57">
         <f>'[2]FTR Finished Product'!$F$195</f>
@@ -36347,7 +36349,7 @@
       </c>
       <c r="L42" s="122">
         <f>(L2+L8+L16+L24+L31+L36)/5</f>
-        <v>0.79365079365079372</v>
+        <v>0.71568627450980382</v>
       </c>
       <c r="M42" s="122">
         <f t="shared" ref="M42" si="1">(M2+M8+M16+M24+M31+M36)/6</f>
@@ -36402,19 +36404,19 @@
       </c>
       <c r="L43" s="144">
         <f>AVERAGE($C$42:L42)</f>
-        <v>0.72257176178035976</v>
+        <v>0.71477530986626081</v>
       </c>
       <c r="M43" s="144">
         <f>AVERAGE($C$42:M42)</f>
-        <v>0.72799863137924592</v>
+        <v>0.72091094782097409</v>
       </c>
       <c r="N43" s="144">
         <f>AVERAGE($C$42:N42)</f>
-        <v>0.73118823094800878</v>
+        <v>0.72469118768625973</v>
       </c>
       <c r="O43" s="143">
         <f t="shared" ref="O43" si="2">AVERAGE(L42,M42,N42,O42,K42)</f>
-        <v>0.75883231886150437</v>
+        <v>0.74323941503330648</v>
       </c>
     </row>
     <row r="44" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Upload 4 files via dashboard admin
- Gross_Efficiency_2026.xlsx
- October_26_Utilities_Tracking.xlsx
- FTR Calculations 2026.xlsx
- October'26 Daily Process Report 2026.xlsx
</commit_message>
<xml_diff>
--- a/data/raw/FTR Calculations 2026.xlsx
+++ b/data/raw/FTR Calculations 2026.xlsx
@@ -9,7 +9,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\FTR Manufacturing- 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{598F05B7-9B53-4053-8613-37E67DED7FD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{209A3550-A2F1-4009-B963-A9ACDA37F9BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="601" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21995,13 +21995,13 @@
             <v>1</v>
           </cell>
           <cell r="E1752">
-            <v>0.41176470588235292</v>
+            <v>0.5</v>
           </cell>
           <cell r="G1752">
-            <v>0.93333333333333335</v>
+            <v>0.94736842105263153</v>
           </cell>
           <cell r="I1752">
-            <v>0.41176470588235292</v>
+            <v>0.5</v>
           </cell>
         </row>
       </sheetData>
@@ -22088,22 +22088,22 @@
         </row>
         <row r="505">
           <cell r="D505">
-            <v>0.83333333333333337</v>
+            <v>0.7142857142857143</v>
           </cell>
           <cell r="G505">
             <v>1</v>
           </cell>
-          <cell r="I505" t="e">
-            <v>#DIV/0!</v>
+          <cell r="I505">
+            <v>1</v>
           </cell>
           <cell r="K505">
             <v>1</v>
           </cell>
           <cell r="M505">
-            <v>0.75</v>
+            <v>0.8</v>
           </cell>
           <cell r="P505">
-            <v>0.5</v>
+            <v>0.6</v>
           </cell>
         </row>
       </sheetData>
@@ -22346,18 +22346,18 @@
             <v>0.88888888888888884</v>
           </cell>
         </row>
-        <row r="631">
-          <cell r="D631">
+        <row r="632">
+          <cell r="D632">
             <v>1</v>
           </cell>
-          <cell r="F631">
-            <v>0.88888888888888884</v>
-          </cell>
-          <cell r="H631">
+          <cell r="F632">
+            <v>0.94444444444444442</v>
+          </cell>
+          <cell r="H632">
             <v>1</v>
           </cell>
-          <cell r="L631">
-            <v>0.88888888888888884</v>
+          <cell r="L632">
+            <v>0.94444444444444442</v>
           </cell>
         </row>
       </sheetData>
@@ -22520,7 +22520,7 @@
             <v>1</v>
           </cell>
           <cell r="F624">
-            <v>0.77777777777777779</v>
+            <v>0.88888888888888884</v>
           </cell>
           <cell r="H624">
             <v>1</v>
@@ -22529,7 +22529,7 @@
             <v>1</v>
           </cell>
           <cell r="L624">
-            <v>0.77777777777777779</v>
+            <v>0.88888888888888884</v>
           </cell>
         </row>
       </sheetData>
@@ -34384,7 +34384,7 @@
       </c>
       <c r="L2" s="51">
         <f>'[1]FTR Brewhouse'!$I$1752</f>
-        <v>0.41176470588235292</v>
+        <v>0.5</v>
       </c>
       <c r="M2" s="51">
         <f>'[2]FTR Brewhouse'!$I$504</f>
@@ -34504,7 +34504,7 @@
       </c>
       <c r="L4" s="54">
         <f>'[1]FTR Brewhouse'!$E$1752</f>
-        <v>0.41176470588235292</v>
+        <v>0.5</v>
       </c>
       <c r="M4" s="54">
         <f>'[2]FTR Brewhouse'!$E$504</f>
@@ -34564,7 +34564,7 @@
       </c>
       <c r="L5" s="54">
         <f>'[1]FTR Brewhouse'!$G$1752</f>
-        <v>0.93333333333333335</v>
+        <v>0.94736842105263153</v>
       </c>
       <c r="M5" s="54">
         <f>'[2]FTR Brewhouse'!$G$504</f>
@@ -34671,7 +34671,7 @@
       </c>
       <c r="L8" s="51">
         <f>'[1]FTR Fermentation'!$P$505</f>
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="M8" s="51">
         <f>'[3]FTR Fermentation'!$P$552</f>
@@ -34731,7 +34731,7 @@
       </c>
       <c r="L9" s="54">
         <f>'[1]FTR Fermentation'!$D$505</f>
-        <v>0.83333333333333337</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="M9" s="54">
         <f>'[3]FTR Fermentation'!$D$552</f>
@@ -34911,7 +34911,7 @@
       </c>
       <c r="L12" s="54">
         <f>'[1]FTR Fermentation'!$M$505</f>
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="M12" s="54">
         <f>'[3]FTR Fermentation'!$M$552</f>
@@ -34969,9 +34969,9 @@
         <f>'[1]FTR Fermentation'!$I$457</f>
         <v>1</v>
       </c>
-      <c r="L13" s="54" t="e">
+      <c r="L13" s="54">
         <f>'[1]FTR Fermentation'!$I$505</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="M13" s="54">
         <f>'[3]FTR Fermentation'!$I$552</f>
@@ -35506,8 +35506,8 @@
         <v>0.88888888888888884</v>
       </c>
       <c r="L24" s="51">
-        <f>'[1]FTR Packaging'!$L$631</f>
-        <v>0.88888888888888884</v>
+        <f>'[1]FTR Packaging'!$L$632</f>
+        <v>0.94444444444444442</v>
       </c>
       <c r="M24" s="51">
         <f>'[3]FTR Packaging'!$L$664</f>
@@ -35566,8 +35566,8 @@
         <v>0.90697674418604646</v>
       </c>
       <c r="L25" s="54">
-        <f>'[1]FTR Packaging'!$F$631</f>
-        <v>0.88888888888888884</v>
+        <f>'[1]FTR Packaging'!$F$632</f>
+        <v>0.94444444444444442</v>
       </c>
       <c r="M25" s="54">
         <f>'[3]FTR Packaging'!$F$664</f>
@@ -35626,7 +35626,7 @@
         <v>1</v>
       </c>
       <c r="L26" s="54">
-        <f>'[1]FTR Packaging'!$D$631</f>
+        <f>'[1]FTR Packaging'!$D$632</f>
         <v>1</v>
       </c>
       <c r="M26" s="54">
@@ -35686,7 +35686,7 @@
         <v>1</v>
       </c>
       <c r="L27" s="52">
-        <f>'[1]FTR Packaging'!$H$631</f>
+        <f>'[1]FTR Packaging'!$H$632</f>
         <v>1</v>
       </c>
       <c r="M27" s="52">
@@ -35746,8 +35746,8 @@
         <v>0.88888888888888884</v>
       </c>
       <c r="L28" s="52">
-        <f>'[1]FTR Packaging'!$L$631</f>
-        <v>0.88888888888888884</v>
+        <f>'[1]FTR Packaging'!$L$632</f>
+        <v>0.94444444444444442</v>
       </c>
       <c r="M28" s="52">
         <f>'[3]FTR Packaging'!$L$664</f>
@@ -36046,7 +36046,7 @@
       </c>
       <c r="L36" s="51">
         <f>'[1]FTR Finished Product'!$L$624</f>
-        <v>0.77777777777777779</v>
+        <v>0.88888888888888884</v>
       </c>
       <c r="M36" s="51">
         <f>'[2]FTR Finished Product'!$L$195</f>
@@ -36166,7 +36166,7 @@
       </c>
       <c r="L38" s="57">
         <f>'[1]FTR Finished Product'!$F$624</f>
-        <v>0.77777777777777779</v>
+        <v>0.88888888888888884</v>
       </c>
       <c r="M38" s="57">
         <f>'[2]FTR Finished Product'!$F$195</f>
@@ -36349,7 +36349,7 @@
       </c>
       <c r="L42" s="122">
         <f>(L2+L8+L16+L24+L31+L36)/5</f>
-        <v>0.71568627450980382</v>
+        <v>0.78666666666666663</v>
       </c>
       <c r="M42" s="122">
         <f t="shared" ref="M42" si="1">(M2+M8+M16+M24+M31+M36)/6</f>
@@ -36404,19 +36404,19 @@
       </c>
       <c r="L43" s="144">
         <f>AVERAGE($C$42:L42)</f>
-        <v>0.71477530986626081</v>
+        <v>0.72187334908194711</v>
       </c>
       <c r="M43" s="144">
         <f>AVERAGE($C$42:M42)</f>
-        <v>0.72091094782097409</v>
+        <v>0.72736371074432526</v>
       </c>
       <c r="N43" s="144">
         <f>AVERAGE($C$42:N42)</f>
-        <v>0.72469118768625973</v>
+        <v>0.7306062203659982</v>
       </c>
       <c r="O43" s="143">
         <f t="shared" ref="O43" si="2">AVERAGE(L42,M42,N42,O42,K42)</f>
-        <v>0.74323941503330648</v>
+        <v>0.75743549346467909</v>
       </c>
     </row>
     <row r="44" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Upload 3 files via dashboard admin
- October'26 Daily Process Report 2026.xlsx
- FTR Calculations 2026.xlsx
- Gross_Efficiency_2026.xlsx
</commit_message>
<xml_diff>
--- a/data/raw/FTR Calculations 2026.xlsx
+++ b/data/raw/FTR Calculations 2026.xlsx
@@ -9,7 +9,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\FTR Manufacturing- 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6812E064-A649-4C63-BDF4-5351F7508C99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2A9CF5E-0698-4EC3-B394-6F7AF5D022E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="601" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1642,7 +1642,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="167">
+  <cellXfs count="168">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2038,6 +2038,10 @@
     </xf>
     <xf numFmtId="1" fontId="25" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="9" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -21917,11 +21921,12 @@
       <sheetName val="Chart1"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
       <sheetData sheetId="6">
         <row r="172">
           <cell r="I172">
@@ -21991,16 +21996,16 @@
         </row>
         <row r="1752">
           <cell r="C1752">
-            <v>1</v>
+            <v>0.9642857142857143</v>
           </cell>
           <cell r="E1752">
-            <v>0.5</v>
+            <v>0.4107142857142857</v>
           </cell>
           <cell r="G1752">
-            <v>0.94736842105263153</v>
+            <v>0.96153846153846156</v>
           </cell>
           <cell r="I1752">
-            <v>0.5</v>
+            <v>0.39285714285714285</v>
           </cell>
         </row>
       </sheetData>
@@ -22087,7 +22092,7 @@
         </row>
         <row r="505">
           <cell r="D505">
-            <v>0.7142857142857143</v>
+            <v>0.72727272727272729</v>
           </cell>
           <cell r="G505">
             <v>1</v>
@@ -22099,14 +22104,14 @@
             <v>1</v>
           </cell>
           <cell r="M505">
-            <v>0.83333333333333337</v>
+            <v>0.8571428571428571</v>
           </cell>
           <cell r="P505">
-            <v>0.66666666666666663</v>
+            <v>0.7142857142857143</v>
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="8"/>
+      <sheetData sheetId="8" refreshError="1"/>
       <sheetData sheetId="9">
         <row r="515">
           <cell r="D515">
@@ -22532,7 +22537,8 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="12"/>
+      <sheetData sheetId="12" refreshError="1"/>
+      <sheetData sheetId="13" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -28665,7 +28671,7 @@
         <f>'[12]FTR Brewhouse'!$C$846</f>
         <v>0.72602739726027399</v>
       </c>
-      <c r="E3" s="156"/>
+      <c r="E3" s="157"/>
     </row>
     <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -28678,7 +28684,7 @@
         <f>'[12]FTR Brewhouse'!$E$846</f>
         <v>0.9178082191780822</v>
       </c>
-      <c r="E4" s="156"/>
+      <c r="E4" s="157"/>
     </row>
     <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
@@ -28860,7 +28866,7 @@
         <f>'[12]FTR Packaging'!$F$458</f>
         <v>0.65</v>
       </c>
-      <c r="E21" s="156"/>
+      <c r="E21" s="157"/>
     </row>
     <row r="22" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
@@ -28873,13 +28879,13 @@
         <f>'[12]FTR Packaging'!$D$458</f>
         <v>1</v>
       </c>
-      <c r="E22" s="156"/>
+      <c r="E22" s="157"/>
     </row>
     <row r="23" spans="1:6" ht="3.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
       <c r="B23" s="8"/>
       <c r="C23" s="53"/>
-      <c r="E23" s="156"/>
+      <c r="E23" s="157"/>
     </row>
     <row r="24" spans="1:6" ht="3.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7"/>
@@ -29048,7 +29054,7 @@
         <f>'[12]FTR Brewhouse'!$C$1015</f>
         <v>0.87857142857142856</v>
       </c>
-      <c r="E3" s="156"/>
+      <c r="E3" s="157"/>
     </row>
     <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -29061,7 +29067,7 @@
         <f>'[12]FTR Brewhouse'!$E$1015</f>
         <v>0.90714285714285714</v>
       </c>
-      <c r="E4" s="156"/>
+      <c r="E4" s="157"/>
     </row>
     <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
@@ -29243,7 +29249,7 @@
         <f>'[12]FTR Packaging'!$F$553</f>
         <v>0.61904761904761907</v>
       </c>
-      <c r="E21" s="156"/>
+      <c r="E21" s="157"/>
     </row>
     <row r="22" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
@@ -29256,13 +29262,13 @@
         <f>'[12]FTR Packaging'!$D$553</f>
         <v>1</v>
       </c>
-      <c r="E22" s="156"/>
+      <c r="E22" s="157"/>
     </row>
     <row r="23" spans="1:5" ht="3.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
       <c r="B23" s="8"/>
       <c r="C23" s="53"/>
-      <c r="E23" s="156"/>
+      <c r="E23" s="157"/>
     </row>
     <row r="24" spans="1:5" ht="3.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7"/>
@@ -29428,7 +29434,7 @@
         <f>'[12]FTR Brewhouse'!$C$1569</f>
         <v>0.85046728971962615</v>
       </c>
-      <c r="E3" s="156"/>
+      <c r="E3" s="157"/>
     </row>
     <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -29441,7 +29447,7 @@
         <f>'[12]FTR Brewhouse'!$E$1569</f>
         <v>0.85981308411214952</v>
       </c>
-      <c r="E4" s="156"/>
+      <c r="E4" s="157"/>
     </row>
     <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
@@ -29644,7 +29650,7 @@
       <c r="A24" s="7"/>
       <c r="B24" s="8"/>
       <c r="C24" s="53"/>
-      <c r="E24" s="156"/>
+      <c r="E24" s="157"/>
     </row>
     <row r="25" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
@@ -29656,7 +29662,7 @@
       <c r="C25" s="108">
         <v>0.71599999999999997</v>
       </c>
-      <c r="E25" s="156"/>
+      <c r="E25" s="157"/>
     </row>
     <row r="26" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
@@ -29668,7 +29674,7 @@
       <c r="C26" s="54">
         <v>1</v>
       </c>
-      <c r="E26" s="156"/>
+      <c r="E26" s="157"/>
     </row>
     <row r="27" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
@@ -29680,7 +29686,7 @@
       <c r="C27" s="54">
         <v>0.71599999999999997</v>
       </c>
-      <c r="E27" s="156"/>
+      <c r="E27" s="157"/>
     </row>
     <row r="28" spans="1:5" ht="3.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="7"/>
@@ -29809,7 +29815,7 @@
         <f>'[13]FTR Brewhouse'!$C$3240</f>
         <v>0.80132450331125826</v>
       </c>
-      <c r="E3" s="156"/>
+      <c r="E3" s="157"/>
     </row>
     <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -29822,7 +29828,7 @@
         <f>'[13]FTR Brewhouse'!$E$3240</f>
         <v>0.50993377483443714</v>
       </c>
-      <c r="E4" s="156"/>
+      <c r="E4" s="157"/>
     </row>
     <row r="5" spans="1:5" ht="3.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7"/>
@@ -30038,7 +30044,7 @@
         <f>'[13]FTR Packaging'!$F$1344</f>
         <v>0.90384615384615385</v>
       </c>
-      <c r="E24" s="156"/>
+      <c r="E24" s="157"/>
     </row>
     <row r="25" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
@@ -30051,7 +30057,7 @@
         <f>'[13]FTR Packaging'!$D$1344</f>
         <v>0.96491228070175439</v>
       </c>
-      <c r="E25" s="156"/>
+      <c r="E25" s="157"/>
     </row>
     <row r="26" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
@@ -30064,13 +30070,13 @@
         <f>'[13]FTR Packaging'!$H$1344</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E26" s="156"/>
+      <c r="E26" s="157"/>
     </row>
     <row r="27" spans="1:5" ht="3.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7"/>
       <c r="B27" s="8"/>
       <c r="C27" s="9"/>
-      <c r="E27" s="156"/>
+      <c r="E27" s="157"/>
     </row>
     <row r="28" spans="1:5" ht="3.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
@@ -30230,7 +30236,7 @@
         <f>'[13]FTR Brewhouse'!$C$3401</f>
         <v>0.91176470588235292</v>
       </c>
-      <c r="E3" s="156"/>
+      <c r="E3" s="157"/>
     </row>
     <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -30243,7 +30249,7 @@
         <f>'[13]FTR Brewhouse'!$E$3401</f>
         <v>0.88970588235294112</v>
       </c>
-      <c r="E4" s="156"/>
+      <c r="E4" s="157"/>
     </row>
     <row r="5" spans="1:5" ht="3.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7"/>
@@ -30455,7 +30461,7 @@
         <f>'[13]FTR Packaging'!$F$1422</f>
         <v>0.84905660377358494</v>
       </c>
-      <c r="E24" s="156"/>
+      <c r="E24" s="157"/>
     </row>
     <row r="25" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
@@ -30468,7 +30474,7 @@
         <f>'[13]FTR Packaging'!$D$1422</f>
         <v>1</v>
       </c>
-      <c r="E25" s="156"/>
+      <c r="E25" s="157"/>
     </row>
     <row r="26" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
@@ -30481,13 +30487,13 @@
         <f>'[13]FTR Packaging'!$H$1422</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E26" s="156"/>
+      <c r="E26" s="157"/>
     </row>
     <row r="27" spans="1:5" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7"/>
       <c r="B27" s="8"/>
       <c r="C27" s="9"/>
-      <c r="E27" s="156"/>
+      <c r="E27" s="157"/>
     </row>
     <row r="28" spans="1:5" ht="3.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
@@ -31330,7 +31336,7 @@
       </c>
     </row>
     <row r="4" spans="1:38" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="157" t="s">
+      <c r="A4" s="158" t="s">
         <v>59</v>
       </c>
       <c r="B4" s="27" t="s">
@@ -31397,7 +31403,7 @@
       </c>
     </row>
     <row r="5" spans="1:38" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="158"/>
+      <c r="A5" s="159"/>
       <c r="B5" s="113" t="s">
         <v>87</v>
       </c>
@@ -31460,22 +31466,22 @@
         <f>(Table1[[#This Row],[Overall]]-Table1[[#This Row],[TARGET]])*100</f>
         <v>#REF!</v>
       </c>
-      <c r="T5" s="161"/>
-      <c r="U5" s="161"/>
-      <c r="V5" s="161"/>
-      <c r="W5" s="161"/>
-      <c r="X5" s="161"/>
-      <c r="Y5" s="161"/>
-      <c r="Z5" s="161"/>
-      <c r="AA5" s="161"/>
-      <c r="AB5" s="161"/>
-      <c r="AC5" s="161"/>
-      <c r="AD5" s="161"/>
-      <c r="AE5" s="161"/>
-      <c r="AF5" s="161"/>
+      <c r="T5" s="162"/>
+      <c r="U5" s="162"/>
+      <c r="V5" s="162"/>
+      <c r="W5" s="162"/>
+      <c r="X5" s="162"/>
+      <c r="Y5" s="162"/>
+      <c r="Z5" s="162"/>
+      <c r="AA5" s="162"/>
+      <c r="AB5" s="162"/>
+      <c r="AC5" s="162"/>
+      <c r="AD5" s="162"/>
+      <c r="AE5" s="162"/>
+      <c r="AF5" s="162"/>
     </row>
     <row r="6" spans="1:38" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="159"/>
+      <c r="A6" s="160"/>
       <c r="B6" s="109" t="s">
         <v>88</v>
       </c>
@@ -31529,7 +31535,7 @@
       <c r="AF6" s="106"/>
     </row>
     <row r="7" spans="1:38" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="162" t="s">
+      <c r="A7" s="163" t="s">
         <v>60</v>
       </c>
       <c r="B7" s="27" t="s">
@@ -31596,7 +31602,7 @@
       </c>
     </row>
     <row r="8" spans="1:38" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="162"/>
+      <c r="A8" s="163"/>
       <c r="B8" s="28" t="s">
         <v>3</v>
       </c>
@@ -31661,7 +31667,7 @@
       </c>
     </row>
     <row r="9" spans="1:38" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="162"/>
+      <c r="A9" s="163"/>
       <c r="B9" s="27" t="s">
         <v>4</v>
       </c>
@@ -31726,7 +31732,7 @@
       </c>
     </row>
     <row r="10" spans="1:38" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="162"/>
+      <c r="A10" s="163"/>
       <c r="B10" s="28" t="s">
         <v>5</v>
       </c>
@@ -31791,7 +31797,7 @@
       </c>
     </row>
     <row r="11" spans="1:38" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="162"/>
+      <c r="A11" s="163"/>
       <c r="B11" s="113" t="s">
         <v>7</v>
       </c>
@@ -31854,21 +31860,21 @@
         <f>(Table1[[#This Row],[Overall]]-Table1[[#This Row],[TARGET]])*100</f>
         <v>#REF!</v>
       </c>
-      <c r="T11" s="161" t="s">
+      <c r="T11" s="162" t="s">
         <v>82</v>
       </c>
-      <c r="U11" s="161"/>
-      <c r="V11" s="161"/>
-      <c r="W11" s="161"/>
-      <c r="X11" s="161"/>
-      <c r="Y11" s="161"/>
-      <c r="Z11" s="161"/>
-      <c r="AA11" s="161"/>
-      <c r="AB11" s="161"/>
-      <c r="AC11" s="161"/>
-      <c r="AD11" s="161"/>
-      <c r="AE11" s="161"/>
-      <c r="AF11" s="161"/>
+      <c r="U11" s="162"/>
+      <c r="V11" s="162"/>
+      <c r="W11" s="162"/>
+      <c r="X11" s="162"/>
+      <c r="Y11" s="162"/>
+      <c r="Z11" s="162"/>
+      <c r="AA11" s="162"/>
+      <c r="AB11" s="162"/>
+      <c r="AC11" s="162"/>
+      <c r="AD11" s="162"/>
+      <c r="AE11" s="162"/>
+      <c r="AF11" s="162"/>
       <c r="AG11" s="105"/>
       <c r="AH11" s="105"/>
       <c r="AI11" s="105"/>
@@ -31877,7 +31883,7 @@
       <c r="AL11" s="105"/>
     </row>
     <row r="12" spans="1:38" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="163" t="s">
+      <c r="A12" s="164" t="s">
         <v>56</v>
       </c>
       <c r="B12" s="111" t="s">
@@ -31944,7 +31950,7 @@
       </c>
     </row>
     <row r="13" spans="1:38" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="163"/>
+      <c r="A13" s="164"/>
       <c r="B13" s="113" t="s">
         <v>10</v>
       </c>
@@ -32007,24 +32013,24 @@
         <f>(Table1[[#This Row],[Overall]]-Table1[[#This Row],[TARGET]])*100</f>
         <v>#REF!</v>
       </c>
-      <c r="T13" s="161" t="s">
+      <c r="T13" s="162" t="s">
         <v>85</v>
       </c>
-      <c r="U13" s="161"/>
-      <c r="V13" s="161"/>
-      <c r="W13" s="161"/>
-      <c r="X13" s="161"/>
-      <c r="Y13" s="161"/>
-      <c r="Z13" s="161"/>
-      <c r="AA13" s="161"/>
-      <c r="AB13" s="161"/>
-      <c r="AC13" s="161"/>
-      <c r="AD13" s="161"/>
-      <c r="AE13" s="161"/>
-      <c r="AF13" s="161"/>
+      <c r="U13" s="162"/>
+      <c r="V13" s="162"/>
+      <c r="W13" s="162"/>
+      <c r="X13" s="162"/>
+      <c r="Y13" s="162"/>
+      <c r="Z13" s="162"/>
+      <c r="AA13" s="162"/>
+      <c r="AB13" s="162"/>
+      <c r="AC13" s="162"/>
+      <c r="AD13" s="162"/>
+      <c r="AE13" s="162"/>
+      <c r="AF13" s="162"/>
     </row>
     <row r="14" spans="1:38" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="163"/>
+      <c r="A14" s="164"/>
       <c r="B14" s="111" t="s">
         <v>13</v>
       </c>
@@ -32089,7 +32095,7 @@
       </c>
     </row>
     <row r="15" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="163"/>
+      <c r="A15" s="164"/>
       <c r="B15" s="111" t="s">
         <v>14</v>
       </c>
@@ -32136,7 +32142,7 @@
       </c>
     </row>
     <row r="16" spans="1:38" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="164" t="s">
+      <c r="A16" s="165" t="s">
         <v>61</v>
       </c>
       <c r="B16" s="113" t="s">
@@ -32201,24 +32207,24 @@
         <f>(Table1[[#This Row],[Overall]]-Table1[[#This Row],[TARGET]])*100</f>
         <v>#REF!</v>
       </c>
-      <c r="T16" s="160" t="s">
+      <c r="T16" s="161" t="s">
         <v>83</v>
       </c>
-      <c r="U16" s="160"/>
-      <c r="V16" s="160"/>
-      <c r="W16" s="160"/>
-      <c r="X16" s="160"/>
-      <c r="Y16" s="160"/>
-      <c r="Z16" s="160"/>
-      <c r="AA16" s="160"/>
-      <c r="AB16" s="160"/>
-      <c r="AC16" s="160"/>
-      <c r="AD16" s="160"/>
-      <c r="AE16" s="160"/>
-      <c r="AF16" s="160"/>
+      <c r="U16" s="161"/>
+      <c r="V16" s="161"/>
+      <c r="W16" s="161"/>
+      <c r="X16" s="161"/>
+      <c r="Y16" s="161"/>
+      <c r="Z16" s="161"/>
+      <c r="AA16" s="161"/>
+      <c r="AB16" s="161"/>
+      <c r="AC16" s="161"/>
+      <c r="AD16" s="161"/>
+      <c r="AE16" s="161"/>
+      <c r="AF16" s="161"/>
     </row>
     <row r="17" spans="1:32" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="164"/>
+      <c r="A17" s="165"/>
       <c r="B17" s="111" t="s">
         <v>19</v>
       </c>
@@ -32283,7 +32289,7 @@
       </c>
     </row>
     <row r="18" spans="1:32" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="164" t="s">
+      <c r="A18" s="165" t="s">
         <v>57</v>
       </c>
       <c r="B18" s="111" t="s">
@@ -32350,7 +32356,7 @@
       </c>
     </row>
     <row r="19" spans="1:32" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="164"/>
+      <c r="A19" s="165"/>
       <c r="B19" s="111" t="s">
         <v>24</v>
       </c>
@@ -32415,7 +32421,7 @@
       </c>
     </row>
     <row r="20" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="165" t="s">
+      <c r="A20" s="166" t="s">
         <v>58</v>
       </c>
       <c r="B20" s="113" t="s">
@@ -32480,22 +32486,22 @@
         <f>(Table1[[#This Row],[Overall]]-Table1[[#This Row],[TARGET]])*100</f>
         <v>#REF!</v>
       </c>
-      <c r="T20" s="161"/>
-      <c r="U20" s="161"/>
-      <c r="V20" s="161"/>
-      <c r="W20" s="161"/>
-      <c r="X20" s="161"/>
-      <c r="Y20" s="161"/>
-      <c r="Z20" s="161"/>
-      <c r="AA20" s="161"/>
-      <c r="AB20" s="161"/>
-      <c r="AC20" s="161"/>
-      <c r="AD20" s="161"/>
-      <c r="AE20" s="161"/>
-      <c r="AF20" s="161"/>
+      <c r="T20" s="162"/>
+      <c r="U20" s="162"/>
+      <c r="V20" s="162"/>
+      <c r="W20" s="162"/>
+      <c r="X20" s="162"/>
+      <c r="Y20" s="162"/>
+      <c r="Z20" s="162"/>
+      <c r="AA20" s="162"/>
+      <c r="AB20" s="162"/>
+      <c r="AC20" s="162"/>
+      <c r="AD20" s="162"/>
+      <c r="AE20" s="162"/>
+      <c r="AF20" s="162"/>
     </row>
     <row r="21" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="165"/>
+      <c r="A21" s="166"/>
       <c r="B21" s="111" t="s">
         <v>26</v>
       </c>
@@ -32560,7 +32566,7 @@
       </c>
     </row>
     <row r="22" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="165"/>
+      <c r="A22" s="166"/>
       <c r="B22" s="111" t="s">
         <v>9</v>
       </c>
@@ -32625,7 +32631,7 @@
       </c>
     </row>
     <row r="23" spans="1:32" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="166"/>
+      <c r="A23" s="167"/>
       <c r="B23" s="113" t="s">
         <v>20</v>
       </c>
@@ -34382,7 +34388,7 @@
       </c>
       <c r="L2" s="51">
         <f>'[1]FTR Brewhouse'!$I$1752</f>
-        <v>0.5</v>
+        <v>0.39285714285714285</v>
       </c>
       <c r="M2" s="51">
         <f>'[2]FTR Brewhouse'!$I$504</f>
@@ -34442,7 +34448,7 @@
       </c>
       <c r="L3" s="52">
         <f>'[1]FTR Brewhouse'!$C$1752</f>
-        <v>1</v>
+        <v>0.9642857142857143</v>
       </c>
       <c r="M3" s="52">
         <f>'[2]FTR Brewhouse'!$C$504</f>
@@ -34502,7 +34508,7 @@
       </c>
       <c r="L4" s="54">
         <f>'[1]FTR Brewhouse'!$E$1752</f>
-        <v>0.5</v>
+        <v>0.4107142857142857</v>
       </c>
       <c r="M4" s="54">
         <f>'[2]FTR Brewhouse'!$E$504</f>
@@ -34562,7 +34568,7 @@
       </c>
       <c r="L5" s="54">
         <f>'[1]FTR Brewhouse'!$G$1752</f>
-        <v>0.94736842105263153</v>
+        <v>0.96153846153846156</v>
       </c>
       <c r="M5" s="54">
         <f>'[2]FTR Brewhouse'!$G$504</f>
@@ -34669,7 +34675,7 @@
       </c>
       <c r="L8" s="51">
         <f>'[1]FTR Fermentation'!$P$505</f>
-        <v>0.66666666666666663</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="M8" s="51">
         <f>'[3]FTR Fermentation'!$P$552</f>
@@ -34729,7 +34735,7 @@
       </c>
       <c r="L9" s="54">
         <f>'[1]FTR Fermentation'!$D$505</f>
-        <v>0.7142857142857143</v>
+        <v>0.72727272727272729</v>
       </c>
       <c r="M9" s="54">
         <f>'[3]FTR Fermentation'!$D$552</f>
@@ -34909,7 +34915,7 @@
       </c>
       <c r="L12" s="54">
         <f>'[1]FTR Fermentation'!$M$505</f>
-        <v>0.83333333333333337</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="M12" s="54">
         <f>'[3]FTR Fermentation'!$M$552</f>
@@ -35851,7 +35857,9 @@
       <c r="K31" s="51">
         <v>0.85</v>
       </c>
-      <c r="L31" s="51"/>
+      <c r="L31" s="156">
+        <v>0.85</v>
+      </c>
       <c r="M31" s="51">
         <v>0.79859999999999998</v>
       </c>
@@ -36346,8 +36354,8 @@
         <v>0.77191245450110701</v>
       </c>
       <c r="L42" s="122">
-        <f>(L2+L8+L16+L24+L31+L36)/5</f>
-        <v>0.80175438596491211</v>
+        <f>(L2+L8+L16+L24+L31+L36)/6</f>
+        <v>0.79987468671679196</v>
       </c>
       <c r="M42" s="122">
         <f t="shared" ref="M42" si="1">(M2+M8+M16+M24+M31+M36)/6</f>
@@ -36402,19 +36410,19 @@
       </c>
       <c r="L43" s="144">
         <f>AVERAGE($C$42:L42)</f>
-        <v>0.72338212101177168</v>
+        <v>0.72319415108695961</v>
       </c>
       <c r="M43" s="144">
         <f>AVERAGE($C$42:M42)</f>
-        <v>0.72873532158962029</v>
+        <v>0.72856443983979124</v>
       </c>
       <c r="N43" s="144">
         <f>AVERAGE($C$42:N42)</f>
-        <v>0.73186353030751861</v>
+        <v>0.73170688870350864</v>
       </c>
       <c r="O43" s="143">
         <f t="shared" ref="O43" si="2">AVERAGE(L42,M42,N42,O42,K42)</f>
-        <v>0.76045303732432812</v>
+        <v>0.76007709747470398</v>
       </c>
     </row>
     <row r="44" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -36697,7 +36705,7 @@
       <c r="C3" s="14">
         <v>94.9</v>
       </c>
-      <c r="E3" s="156" t="s">
+      <c r="E3" s="157" t="s">
         <v>32</v>
       </c>
     </row>
@@ -36711,7 +36719,7 @@
       <c r="C4" s="16">
         <v>94.9</v>
       </c>
-      <c r="E4" s="156"/>
+      <c r="E4" s="157"/>
     </row>
     <row r="5" spans="1:5" ht="3.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7"/>
@@ -36912,7 +36920,7 @@
       <c r="C24" s="3">
         <v>70</v>
       </c>
-      <c r="E24" s="156" t="s">
+      <c r="E24" s="157" t="s">
         <v>33</v>
       </c>
     </row>
@@ -36926,7 +36934,7 @@
       <c r="C25" s="6">
         <v>88.9</v>
       </c>
-      <c r="E25" s="156"/>
+      <c r="E25" s="157"/>
     </row>
     <row r="26" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
@@ -36938,7 +36946,7 @@
       <c r="C26" s="6">
         <v>88.9</v>
       </c>
-      <c r="E26" s="156"/>
+      <c r="E26" s="157"/>
     </row>
     <row r="27" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
@@ -36950,13 +36958,13 @@
       <c r="C27" s="6">
         <v>88.9</v>
       </c>
-      <c r="E27" s="156"/>
+      <c r="E27" s="157"/>
     </row>
     <row r="28" spans="1:5" ht="3.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
       <c r="B28" s="8"/>
       <c r="C28" s="9"/>
-      <c r="E28" s="156"/>
+      <c r="E28" s="157"/>
     </row>
     <row r="29" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
@@ -36966,7 +36974,7 @@
       <c r="C29" s="14">
         <v>70</v>
       </c>
-      <c r="E29" s="156"/>
+      <c r="E29" s="157"/>
     </row>
     <row r="30" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">

</xml_diff>

<commit_message>
Upload 6 files via dashboard admin
- October'26 Daily Process Report 2026.xlsx
- October_26_Utilities_Tracking.xlsx
- Gross_Efficiency_2026.xlsx
- October_2026.xls
- FTR Calculations 2026.xlsx
- Finished PM Compliance.xlsx
</commit_message>
<xml_diff>
--- a/data/raw/FTR Calculations 2026.xlsx
+++ b/data/raw/FTR Calculations 2026.xlsx
@@ -9,7 +9,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\FTR Manufacturing- 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6990FDF-4378-42F3-BFFE-2B68BA54B35C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB05474A-1EB8-42ED-A2A1-865CE1EF9925}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="601" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21995,7 +21995,7 @@
         </row>
         <row r="1752">
           <cell r="C1752">
-            <v>0.96491228070175439</v>
+            <v>0.91200000000000003</v>
           </cell>
           <cell r="E1752">
             <v>0.40350877192982454</v>
@@ -22192,24 +22192,24 @@
             <v>0.98571428571428577</v>
           </cell>
         </row>
-        <row r="893">
-          <cell r="D893">
-            <v>0.93846153846153846</v>
-          </cell>
-          <cell r="F893">
+        <row r="899">
+          <cell r="D899">
+            <v>0.95180722891566261</v>
+          </cell>
+          <cell r="F899">
             <v>1</v>
           </cell>
-          <cell r="H893">
-            <v>0.98275862068965514</v>
-          </cell>
-          <cell r="J893">
-            <v>1</v>
-          </cell>
-          <cell r="L893">
-            <v>0.90566037735849059</v>
-          </cell>
-          <cell r="N893">
-            <v>0.79365079365079361</v>
+          <cell r="H899">
+            <v>0.97333333333333338</v>
+          </cell>
+          <cell r="J899">
+            <v>0.98795180722891562</v>
+          </cell>
+          <cell r="L899">
+            <v>0.91549295774647887</v>
+          </cell>
+          <cell r="N899">
+            <v>0.84615384615384615</v>
           </cell>
         </row>
       </sheetData>
@@ -22354,13 +22354,13 @@
             <v>1</v>
           </cell>
           <cell r="F632">
-            <v>0.97499999999999998</v>
+            <v>0.97872340425531912</v>
           </cell>
           <cell r="H632">
             <v>1</v>
           </cell>
           <cell r="L632">
-            <v>0.97435897435897434</v>
+            <v>0.97826086956521741</v>
           </cell>
         </row>
       </sheetData>
@@ -22520,10 +22520,10 @@
         </row>
         <row r="624">
           <cell r="D624">
-            <v>0.9555555555555556</v>
+            <v>0.9642857142857143</v>
           </cell>
           <cell r="F624">
-            <v>0.88372093023255816</v>
+            <v>0.90740740740740744</v>
           </cell>
           <cell r="H624">
             <v>1</v>
@@ -22532,7 +22532,7 @@
             <v>1</v>
           </cell>
           <cell r="L624">
-            <v>0.84444444444444444</v>
+            <v>0.875</v>
           </cell>
         </row>
       </sheetData>
@@ -34446,7 +34446,7 @@
       </c>
       <c r="L3" s="52">
         <f>'[1]FTR Brewhouse'!$C$1752</f>
-        <v>0.96491228070175439</v>
+        <v>0.91200000000000003</v>
       </c>
       <c r="M3" s="52">
         <f>'[2]FTR Brewhouse'!$C$504</f>
@@ -35083,8 +35083,8 @@
         <v>0.98571428571428577</v>
       </c>
       <c r="L16" s="51">
-        <f>'[1]FTR BBT'!$N$893</f>
-        <v>0.79365079365079361</v>
+        <f>'[1]FTR BBT'!$N$899</f>
+        <v>0.84615384615384615</v>
       </c>
       <c r="M16" s="51">
         <f>'[3]FTR BBT'!$N$974</f>
@@ -35143,8 +35143,8 @@
         <v>0.98611111111111116</v>
       </c>
       <c r="L17" s="55">
-        <f>'[1]FTR BBT'!$D$893</f>
-        <v>0.93846153846153846</v>
+        <f>'[1]FTR BBT'!$D$899</f>
+        <v>0.95180722891566261</v>
       </c>
       <c r="M17" s="55">
         <f>'[3]FTR BBT'!$D$974</f>
@@ -35206,8 +35206,8 @@
         <v>1</v>
       </c>
       <c r="L18" s="56">
-        <f>'[1]FTR BBT'!$J$893</f>
-        <v>1</v>
+        <f>'[1]FTR BBT'!$J$899</f>
+        <v>0.98795180722891562</v>
       </c>
       <c r="M18" s="56">
         <f>'[3]FTR BBT'!$J$974</f>
@@ -35266,8 +35266,8 @@
         <v>1</v>
       </c>
       <c r="L19" s="55">
-        <f>'[1]FTR BBT'!$H$893</f>
-        <v>0.98275862068965514</v>
+        <f>'[1]FTR BBT'!$H$899</f>
+        <v>0.97333333333333338</v>
       </c>
       <c r="M19" s="55">
         <f>'[3]FTR BBT'!$H$974</f>
@@ -35326,7 +35326,7 @@
         <v>1</v>
       </c>
       <c r="L20" s="55">
-        <f>'[1]FTR BBT'!$F$893</f>
+        <f>'[1]FTR BBT'!$F$899</f>
         <v>1</v>
       </c>
       <c r="M20" s="55">
@@ -35386,8 +35386,8 @@
         <v>1</v>
       </c>
       <c r="L21" s="52">
-        <f>'[1]FTR BBT'!$L$893</f>
-        <v>0.90566037735849059</v>
+        <f>'[1]FTR BBT'!$L$899</f>
+        <v>0.91549295774647887</v>
       </c>
       <c r="M21" s="52">
         <f>'[3]FTR BBT'!$L$974</f>
@@ -35509,7 +35509,7 @@
       </c>
       <c r="L24" s="51">
         <f>'[1]FTR Packaging'!$L$632</f>
-        <v>0.97435897435897434</v>
+        <v>0.97826086956521741</v>
       </c>
       <c r="M24" s="51">
         <f>'[3]FTR Packaging'!$L$664</f>
@@ -35569,7 +35569,7 @@
       </c>
       <c r="L25" s="54">
         <f>'[1]FTR Packaging'!$F$632</f>
-        <v>0.97499999999999998</v>
+        <v>0.97872340425531912</v>
       </c>
       <c r="M25" s="54">
         <f>'[3]FTR Packaging'!$F$664</f>
@@ -35749,7 +35749,7 @@
       </c>
       <c r="L28" s="52">
         <f>'[1]FTR Packaging'!$L$632</f>
-        <v>0.97435897435897434</v>
+        <v>0.97826086956521741</v>
       </c>
       <c r="M28" s="52">
         <f>'[3]FTR Packaging'!$L$664</f>
@@ -36050,7 +36050,7 @@
       </c>
       <c r="L36" s="51">
         <f>'[1]FTR Finished Product'!$L$624</f>
-        <v>0.84444444444444444</v>
+        <v>0.875</v>
       </c>
       <c r="M36" s="51">
         <f>'[2]FTR Finished Product'!$L$195</f>
@@ -36170,7 +36170,7 @@
       </c>
       <c r="L38" s="57">
         <f>'[1]FTR Finished Product'!$F$624</f>
-        <v>0.88372093023255816</v>
+        <v>0.90740740740740744</v>
       </c>
       <c r="M38" s="57">
         <f>'[2]FTR Finished Product'!$F$195</f>
@@ -36230,7 +36230,7 @@
       </c>
       <c r="L39" s="57">
         <f>'[1]FTR Finished Product'!$D$624</f>
-        <v>0.9555555555555556</v>
+        <v>0.9642857142857143</v>
       </c>
       <c r="M39" s="57">
         <f>'[2]FTR Finished Product'!$D$195</f>
@@ -36353,7 +36353,7 @@
       </c>
       <c r="L42" s="122">
         <f>(L2+L8+L16+L24+L31+L36)/6</f>
-        <v>0.76045080650343799</v>
+        <v>0.77494422371424665</v>
       </c>
       <c r="M42" s="122">
         <f t="shared" ref="M42" si="1">(M2+M8+M16+M24+M31+M36)/6</f>
@@ -36408,19 +36408,19 @@
       </c>
       <c r="L43" s="144">
         <f>AVERAGE($C$42:L42)</f>
-        <v>0.71925176306562422</v>
+        <v>0.72070110478670513</v>
       </c>
       <c r="M43" s="144">
         <f>AVERAGE($C$42:M42)</f>
-        <v>0.72498045072948625</v>
+        <v>0.72629803411228699</v>
       </c>
       <c r="N43" s="144">
         <f>AVERAGE($C$42:N42)</f>
-        <v>0.72842156535239588</v>
+        <v>0.72962935011996322</v>
       </c>
       <c r="O43" s="143">
         <f t="shared" ref="O43" si="2">AVERAGE(L42,M42,N42,O42,K42)</f>
-        <v>0.75219232143203318</v>
+        <v>0.755091004874195</v>
       </c>
     </row>
     <row r="44" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>